<commit_message>
Updated state-based authoritative links list.
</commit_message>
<xml_diff>
--- a/sources/States_Source_Validation_Links.xlsx
+++ b/sources/States_Source_Validation_Links.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{478D3B54-4D2D-4FD9-8C11-A3192D2B2F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40D8AA2-E9E8-409E-89B6-1482347D93D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9E6F9348-DD40-48E7-B657-955CDE871BDA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9E6F9348-DD40-48E7-B657-955CDE871BDA}"/>
   </bookViews>
   <sheets>
     <sheet name="State Sources" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="147">
   <si>
     <t>State</t>
   </si>
@@ -270,9 +270,6 @@
     <t>Missouri</t>
   </si>
   <si>
-    <t>https://health.mo.gov/living/wellness/nutrition/culinaryskills/pdf/Fruits-and-Vegetables-Harvest-Poster.pdf</t>
-  </si>
-  <si>
     <t>https://columbiafarmersmarket.org/wp-content/uploads/2023/04/SeasonalityChart.png</t>
   </si>
   <si>
@@ -469,6 +466,18 @@
   </si>
   <si>
     <t>https://osse.dc.gov/sites/default/files/dc/sites/osse/service_content/attachments/DCF2S%20seasonality%20chart%202013-web.pdf</t>
+  </si>
+  <si>
+    <t>https://eatlocalfirst.org/wp-content/uploads/2025/04/eat_local_first_seasonality_calendar.pdf</t>
+  </si>
+  <si>
+    <t>https://cms.agr.wa.gov/WSDAKentico/Imported/SeasonalityChartFruitLegumeHerbsfinal.pdf?/SeasonalityChartFruitLegumeHerbsfinal.pdf&amp;_gl=1*3voc4j*_ga*Mzk3MzA0NzkwLjE3NTk4NTM2MDE.*_ga_9JCK8SVQPE*czE3NTk4NTM2MDEkbzEkZzEkdDE3NTk4NTM2NjckajU2JGwwJGgw</t>
+  </si>
+  <si>
+    <t>https://cms.agr.wa.gov/WSDAKentico/Imported/SeasonalityChartHUSSCVegetablefinal.pdf?/SeasonalityChartHUSSCVegetablefinal.pdf&amp;_gl=1*3voc4j*_ga*Mzk3MzA0NzkwLjE3NTk4NTM2MDE.*_ga_9JCK8SVQPE*czE3NTk4NTM2MDEkbzEkZzEkdDE3NTk4NTM2NjckajU2JGwwJGgw</t>
+  </si>
+  <si>
+    <t>https://health.mo.gov/living/wellness/nutrition/farmtopreschool/pdf/harvest-season-calendar.pdf</t>
   </si>
 </sst>
 </file>
@@ -880,45 +889,45 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" t="s">
         <v>113</v>
-      </c>
-      <c r="B4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" t="s">
         <v>127</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>128</v>
-      </c>
-      <c r="C6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -934,7 +943,7 @@
         <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -961,18 +970,18 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B13" t="s">
         <v>120</v>
-      </c>
-      <c r="B13" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1010,13 +1019,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="B17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1029,16 +1038,16 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" t="s">
         <v>81</v>
       </c>
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>82</v>
-      </c>
-      <c r="D19" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1111,43 +1120,46 @@
         <v>76</v>
       </c>
       <c r="B26" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>78</v>
+      <c r="D26" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" t="s">
         <v>104</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>105</v>
-      </c>
-      <c r="C27" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" t="s">
         <v>95</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>96</v>
-      </c>
-      <c r="C28" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" t="s">
         <v>132</v>
       </c>
-      <c r="B29" t="s">
-        <v>133</v>
-      </c>
       <c r="C29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1170,13 +1182,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
+        <v>110</v>
+      </c>
+      <c r="B32" t="s">
+        <v>140</v>
+      </c>
+      <c r="C32" t="s">
         <v>111</v>
-      </c>
-      <c r="B32" t="s">
-        <v>141</v>
-      </c>
-      <c r="C32" t="s">
-        <v>112</v>
       </c>
       <c r="D32" s="1"/>
     </row>
@@ -1200,10 +1212,10 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>101</v>
+      </c>
+      <c r="B35" t="s">
         <v>102</v>
-      </c>
-      <c r="B35" t="s">
-        <v>103</v>
       </c>
       <c r="D35" s="1"/>
     </row>
@@ -1221,23 +1233,23 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B37" s="1"/>
       <c r="C37" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" t="s">
         <v>90</v>
-      </c>
-      <c r="D37" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B38" s="1"/>
       <c r="C38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -1254,7 +1266,7 @@
         <v>30</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D40" s="1"/>
     </row>
@@ -1269,13 +1281,13 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>97</v>
+      </c>
+      <c r="B42" t="s">
         <v>98</v>
       </c>
-      <c r="B42" t="s">
-        <v>99</v>
-      </c>
       <c r="C42" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -1292,33 +1304,33 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" t="s">
         <v>85</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="C44" t="s">
-        <v>88</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>114</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" t="s">
         <v>117</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>118</v>
-      </c>
-      <c r="F45" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -1343,13 +1355,22 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" t="s">
         <v>122</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>123</v>
       </c>
-      <c r="C48" t="s">
-        <v>124</v>
+      <c r="D48" t="s">
+        <v>143</v>
+      </c>
+      <c r="E48" t="s">
+        <v>144</v>
+      </c>
+      <c r="F48" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -1377,23 +1398,23 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>134</v>
+      </c>
+      <c r="B52" t="s">
         <v>135</v>
-      </c>
-      <c r="B52" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>141</v>
+      </c>
+      <c r="B53" t="s">
         <v>142</v>
-      </c>
-      <c r="B53" t="s">
-        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1418,22 +1439,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>